<commit_message>
Sync affiliate_products.xlsx from rocket repo
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="80">
   <si>
     <t>No</t>
   </si>
@@ -103,48 +103,6 @@
     <t>https://s.lazada.co.th/s.Z6hUBK?c=a&amp;t=p-i69orjh-sQEG95F</t>
   </si>
   <si>
-    <t>ลองเข้ามาดู Café Amazon (อาคารสินธร - SD3951) ที่ Shopee! https://spf.shopee.co.th/9pbHxS0Kia</t>
-  </si>
-  <si>
-    <t>ลองเข้ามาดู Punthai Coffee (ซีแพค พระราม7) ที่ Shopee! https://spf.shopee.co.th/4VZlbcIDI7</t>
-  </si>
-  <si>
-    <t>ลองเข้ามาดู The Pizza Company (วงศกร) ที่ Shopee! https://spf.shopee.co.th/6feGBaJAVI</t>
-  </si>
-  <si>
-    <t>ลองเข้ามาดู Subway (เอ็มอาร์ที ลาดพร้าว) ที่ Shopee! https://spf.shopee.co.th/AKXYYIsLV7</t>
-  </si>
-  <si>
-    <t>ลองเข้ามาดู บัณฑิตคิม ข้าวมันไก่ (ลาดพร้าววังหิน) ที่ Shopee! https://spf.shopee.co.th/2qRXcVAmdq</t>
-  </si>
-  <si>
-    <t>ลองเข้ามาดู ขาหมูชานเมือง ข้าวมันไก่ อาหารตามสั่ง ก๋วยเตี๋ยว (รัชดาภิเษก7) ที่ Shopee! https://spf.shopee.co.th/AAE8Lxgj6W</t>
-  </si>
-  <si>
-    <t>ลองเข้ามาดู ข้าวหมูทอดอร่อยมาก (ประชาอุทิศ) ที่ Shopee! https://spf.shopee.co.th/BQmRZCjn6</t>
-  </si>
-  <si>
-    <t>ลองเข้ามาดู Chester's (ปตท. กรุงเทพ-บางแค2 วงแหวน - 107208 ) ที่ Shopee! https://spf.shopee.co.th/9pbHxIUZ3g</t>
-  </si>
-  <si>
-    <t>ลองเข้ามาดู McDonald's (พีทีที บรม ขาออก) ที่ Shopee! https://spf.shopee.co.th/3B4O11yxCV</t>
-  </si>
-  <si>
-    <t>ลองเข้ามาดู KFC (ปตท. กาญจนาภิเษก ตลิ่งชัน) ที่ Shopee! https://spf.shopee.co.th/6L1PmpO0Jy</t>
-  </si>
-  <si>
-    <t>ลองเข้ามาดู Starbucks (โรบินสัน บ้านฉาง) ที่ Shopee! https://spf.shopee.co.th/809dlpHQ2L</t>
-  </si>
-  <si>
-    <t>ลองเข้ามาดู Punthai Coffee (นิคมอุตสาหกรรมมาบตาพุด) ที่ Shopee! https://spf.shopee.co.th/7AaWmGyzrV</t>
-  </si>
-  <si>
-    <t>ลองเข้ามาดู ครัวฅนลาบ.ตำ.สั่ง (ถนนมาบชลูด-แหลมสน) ที่ Shopee! https://spf.shopee.co.th/3qK4o80svV</t>
-  </si>
-  <si>
-    <t>ลองเข้ามาดู Café Amazon (สำนักงานปปง. - SD5580) ที่ Shopee! https://spf.shopee.co.th/40dV0P4yci</t>
-  </si>
-  <si>
     <t>Essager หัวชาร์จ GaN 65W ชาร์จเร็ว Type-C/USB-A 2-in-1</t>
   </si>
   <si>
@@ -173,6 +131,129 @@
   </si>
   <si>
     <t>Baseus โคมไฟตั้งโต๊ะ LED แม่เหล็กไร้สาย Magnetic</t>
+  </si>
+  <si>
+    <t>ลองเข้ามาดู Café Amazon  ที่ Shopee! https://spf.shopee.co.th/40dV0P4yci</t>
+  </si>
+  <si>
+    <t>ลองเข้ามาดู ครัวฅนลาบ.ตำ.สั่ง  ที่ Shopee! https://spf.shopee.co.th/3qK4o80svV</t>
+  </si>
+  <si>
+    <t>ลองเข้ามาดู Punthai Coffee ที่ Shopee! https://spf.shopee.co.th/7AaWmGyzrV</t>
+  </si>
+  <si>
+    <t>ลองเข้ามาดู Starbucks ที่ Shopee! https://spf.shopee.co.th/809dlpHQ2L</t>
+  </si>
+  <si>
+    <t>ลองเข้ามาดู KFC ที่ Shopee! https://spf.shopee.co.th/6L1PmpO0Jy</t>
+  </si>
+  <si>
+    <t>ลองเข้ามาดู McDonald's ที่ Shopee! https://spf.shopee.co.th/3B4O11yxCV</t>
+  </si>
+  <si>
+    <t>ลองเข้ามาดู Chester's ที่ Shopee! https://spf.shopee.co.th/9pbHxIUZ3g</t>
+  </si>
+  <si>
+    <t>ลองเข้ามาดู ข้าวหมูทอดอร่อยมาก ที่ Shopee! https://spf.shopee.co.th/BQmRZCjn6</t>
+  </si>
+  <si>
+    <t>ลองเข้ามาดู ขาหมูชานเมือง ข้าวมันไก่ อาหารตามสั่ง ก๋วยเตี๋ยว ที่ Shopee! https://spf.shopee.co.th/AAE8Lxgj6W</t>
+  </si>
+  <si>
+    <t>ลองเข้ามาดู บัณฑิตคิม ข้าวมันไก่  ที่ Shopee! https://spf.shopee.co.th/2qRXcVAmdq</t>
+  </si>
+  <si>
+    <t>ลองเข้ามาดู Subway ที่ Shopee! https://spf.shopee.co.th/AKXYYIsLV7</t>
+  </si>
+  <si>
+    <t>ลองเข้ามาดู The Pizza Company ที่ Shopee! https://spf.shopee.co.th/6feGBaJAVI</t>
+  </si>
+  <si>
+    <t>ลองเข้ามาดู Punthai Coffee ที่ Shopee! https://spf.shopee.co.th/4VZlbcIDI7</t>
+  </si>
+  <si>
+    <t>ลองเข้ามาดู Café Amazon ที่ Shopee! https://spf.shopee.co.th/9pbHxS0Kia</t>
+  </si>
+  <si>
+    <t>Rojeco เครื่องให้อาหารแมวอัตโนมัติ ปุ่มกด WIFI ควบคุมอัจฉริยะ ขนาด 2 ลิตร</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/2LVKz84rKR</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6po6f?c=a&amp;t=p-i58qIVk-sNeq30B</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6po89?c=a&amp;t=p-i5UANgd-sNC8zX0</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/3qK8m24JRm</t>
+  </si>
+  <si>
+    <t>Dr.Zkin Pet Spray ผลิตภัณฑ์สำหรับสัตว์เลี้ยง บำรุงขน ดับกลิ่น เพิ่มความหอม</t>
+  </si>
+  <si>
+    <t>ใหม่!เซาปิ่งเปี๊ยะนุ่มลาวา สูตรเยาวราช 15 ปี ตัวแป้งทำจากมันเทศ เก็บได้นานเดือน อุ่นเวฟทานได้เรื่อยๆ</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/8AT7w2iCji</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6poow?c=a&amp;t=p-i6YOKrQ-sSFykLR</t>
+  </si>
+  <si>
+    <t>แคบหมูกึ่งสำเร็จรูป (ติดมัน) Pig a Pop แคบหมูแบบทอดเอง แคบหมูป๊อป แคบหมู แคปหมู</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/2g8BO1Iioo</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6poHW?t=p-iHYzWWS-s2EM8tAv</t>
+  </si>
+  <si>
+    <t>(ได้เยอะ จุใจ!! ) สาหร่ายทอดกรอบ กระป๋องใหญ่ 2700ml ปริมาณ145g มีให้เลือก3รส ดั้งเดิม ต้มยำ หม่าล่า</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6poC8?c=b&amp;t=p-i2Xh0Lf-sQBAMgv</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/10zxP54mnK</t>
+  </si>
+  <si>
+    <t>น้ำมันมรกต ขนาด 1 ลิตร สำหรับทำอาหาร แพ็ค 3 ขวด | น้ำมันพืชทำอาหาร ผัด ทอด อเนกประสงค์ ใช้ได้ทุกเมนู</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/7VDR93nl23</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6pL0t?c=b&amp;t=p-i6SvdvJ-sRgXbld</t>
+  </si>
+  <si>
+    <t>[✅โค้ดส่งฟรี+🎫โค้ดคุุ้ม] ปลากระป๋อง ตรา สามแม่ครัว ปลาแมคเคอเรลในซอสมะเขือเทศ 155 กรัม x 8 กระป๋อง ♥ ล็อตใหม่</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6pL38?c=b&amp;t=p-iJ4zNe-sV3TtR</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/809hk3ycB9</t>
+  </si>
+  <si>
+    <t>koreadong โคเรียดอง แซลมอนดองซีอิ๊วเกาหลี 5 กระปุก สุดฮิต แถมฟรีน้ำจิ้ม</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6pL7d?c=a&amp;t=p-i2qXX8u-sAvS9sD</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/809hk8D15m</t>
+  </si>
+  <si>
+    <t>yoyopet : Furry Fresh สเปรย์ปรับอากาศ สเปรย์น้ำหอม ดับกลิ่นฉี่แมวและสัตว์เลี้ยง ปลอดภัย 500ml</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/1LcnnxemB8</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6pLoQ?c=b&amp;t=p-i6XgnuV-sSKIzpC</t>
   </si>
 </sst>
 </file>
@@ -234,7 +315,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -257,12 +338,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBBBBBB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBBBBBB"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -276,6 +368,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -578,7 +673,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -617,7 +712,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>7</v>
@@ -632,7 +727,7 @@
         <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
@@ -640,7 +735,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>11</v>
@@ -655,7 +750,7 @@
         <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
@@ -663,7 +758,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>13</v>
@@ -678,12 +773,12 @@
         <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>15</v>
@@ -698,12 +793,12 @@
         <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>17</v>
@@ -718,12 +813,12 @@
         <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>19</v>
@@ -738,12 +833,12 @@
         <v>10</v>
       </c>
       <c r="G7" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>21</v>
@@ -758,12 +853,12 @@
         <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>23</v>
@@ -778,12 +873,12 @@
         <v>10</v>
       </c>
       <c r="G9" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>25</v>
@@ -798,12 +893,12 @@
         <v>10</v>
       </c>
       <c r="G10" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B11" s="6" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>27</v>
@@ -818,27 +913,172 @@
         <v>10</v>
       </c>
       <c r="G11" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="B12" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>10</v>
+      </c>
       <c r="G12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="B13" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="B14" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="B15" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G15" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G13" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G14" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G15" t="s">
-        <v>42</v>
+    <row r="16" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="B16" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="B17" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="B18" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="B19" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="B20" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -863,6 +1103,24 @@
     <hyperlink ref="D10" r:id="rId18"/>
     <hyperlink ref="C11" r:id="rId19"/>
     <hyperlink ref="D11" r:id="rId20"/>
+    <hyperlink ref="C12" r:id="rId21"/>
+    <hyperlink ref="D12" r:id="rId22"/>
+    <hyperlink ref="D13" r:id="rId23"/>
+    <hyperlink ref="C13" r:id="rId24"/>
+    <hyperlink ref="C14" r:id="rId25"/>
+    <hyperlink ref="D14" r:id="rId26"/>
+    <hyperlink ref="C15" r:id="rId27"/>
+    <hyperlink ref="D15" r:id="rId28"/>
+    <hyperlink ref="D16" r:id="rId29"/>
+    <hyperlink ref="C16" r:id="rId30"/>
+    <hyperlink ref="C17" r:id="rId31"/>
+    <hyperlink ref="D17" r:id="rId32"/>
+    <hyperlink ref="D18" r:id="rId33"/>
+    <hyperlink ref="C18" r:id="rId34"/>
+    <hyperlink ref="D19" r:id="rId35"/>
+    <hyperlink ref="C19" r:id="rId36"/>
+    <hyperlink ref="C20" r:id="rId37"/>
+    <hyperlink ref="D20" r:id="rId38"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Cordless Lawn Mower, Air Bed, and Mobi Garden Chair to affiliate products
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1323,6 +1323,96 @@
       <c r="F20" s="5" t="inlineStr">
         <is>
           <t>ลด 20% วันนี้เท่านั้น</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>【ส่งถึงในวันเดียวกัน】เครื่องตัดหญ้าไฟฟ้า ไร้สาย แบต2ก้อน 50000mah ง่ายต่อการพกพา พับเก็บได้ Lawn mower</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/5L91LfuOyh</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>เครื่องตัดหญ้าไร้สาย พับเก็บได้ พกพาสะดวก</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>เตียงเป่าลม อัตโนมัติ ที่นอนลมกลางแจ้ง พับได้ แบบพกพา พร้อมปั๊มลมในตัว ที่นอนลม แบบหนา 40/25ซม</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/20sZNboI0O</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>ที่นอนลมเป่าลมอัตโนมัติ พับได้ พกพาสะดวก</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>6</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Mobi GARDEN เก้าอี้ปิกนิก พับได้ แบบพกพา สวยหรู สําหรับตั้งแคมป์กลางแจ้ง</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7Ku5jRGwQA</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>เก้าอี้แคมป์ปิ้งพับได้ Mobi Garden พกพาสะดวก</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Ant Gel, Sipeau Tissue, Minimal Sofa, and Masaru Fan to affiliate products
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1413,6 +1413,126 @@
       <c r="F23" t="inlineStr">
         <is>
           <t>เก้าอี้แคมป์ปิ้งพับได้ Mobi Garden พกพาสะดวก</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>7</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>เจลกำจัดมด ANTIANT แอนตี้แอนท์ [ของแท้จากร้าน Antiant Thailand]</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/50WAxOvzHX</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>เจลกำจัดมด แอนตี้แอนท์ ของแท้ กำจัดมดตายยกรัง ปลอดภัยต่อผู้ใช้</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>8</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>5เเพ็ค กระดาษทิชชู่ Sipeau กระดาษทิชชู่คุณภาพสูง นุ่ม กระดาษทิชชู่เช็ดหน้า</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/2LVPmXFuzA</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>กระดาษทิชชู่เช็ดหน้า Sipeau 5 แพ็ค หนานุ่ม ไม่ระคายเคืองผิว</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>9</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>เก้าอี้พักผ่อน Minimal โซฟา ปรับนอนได้ ถึง160°c สีครีม เบาะฟองน้ำหนา10ซม. นุ่มสบาย ผ้ากำมะหยี่</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/5q5HwzecQH</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>เก้าอี้โซฟาปรับนอนได้ 160 องศา สไตล์มินิมอล นุ่มสบาย เหมาะแก่การพักผ่อน</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>10</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>MASARU พัดลมไร้สาย SCFP-910 พัดลม 10นิ้ว พัดลมพกพาไร้สาย พัดลม แบตเตอรี่ แบตลิเธียม 20V</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/1BJSOn3rqU</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>พัดลมพกพาไร้สาย MASARU 10 นิ้ว แบตเตอรี่อึด เย็นสบายทุกที่</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update affiliate products - add white hair shampoo, toothpaste, probiotic, protein, paseo tissues, head & shoulders
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1533,6 +1533,186 @@
       <c r="F27" t="inlineStr">
         <is>
           <t>พัดลมพกพาไร้สาย MASARU 10 นิ้ว แบตเตอรี่อึด เย็นสบายทุกที่</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>11</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>แชมพูปิดผมขาวหอมเกศ พร้อมบำรุงเส้นผม แบบขวด 300 มล.</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/50WEKngBoG</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>แชมพูปิดผมขาวหอมเกศ กลิ่นหอมธรรมชาติ อ่อนโยน บำรุงผมให้นุ่มสลวย</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>12</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ยาสีฟันขิงขิง ยาสีฟันสมุนไพร ลดกลิ่นปาก ฟันขาวแข็งแรง (ซื้อ 1 แถม 1)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/40dh91vVju</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>ยาสีฟันขิงขิง ยาสีฟันสมุนไพรเข้มข้น ลดกลิ่นปากยาวนาน ฟันสะอาดแข็งแรง</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>13</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Life Plus โพรไบโอ18 (Life Plus ProBio18) โพรไบโอติกส์ชนิดกรอกปาก</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8fPWhfELMS</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>โพรไบโอติกส์ Life Plus ProBio18 ช่วยระบบขับถ่ายและสมดุลลำไส้ ชนิดกรอกปากทานง่าย</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>14</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>[แพ็คคู่] Head and Shoulders แชมพูขจัดรังแค สูตรคูล เมนทอล 370 มล. x 2 ขวด</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/6feSK37y2S</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>แชมพู Head &amp; Shoulders คูลเมนทอล แพ็คคู่สุดคุ้ม เย็นสดชื่น สะอาดปราศจากรังแค</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>15</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>[โปร 1 แถม 1] Dr.JiLL JIL S Plant-Based Protein โปรตีนพืชสำหรับผู้ใหญ่ 400 กรัม</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/4Ax7LVYpmM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>โปรตีนพืชสำหรับผู้ใหญ่ JIL S by Dr.Jill ละลายง่าย รสชาติอร่อย สุขภาพดีครบถ้วน</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>16</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>PASEO พาซิโอ เบบี้เพียว ซอฟท์แพ็ค กระดาษเช็ดหน้า หนา 3 ชั้น (ยกลัง 4 ห่อ x 12 แพ็ค)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/6VL27rrtdF</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>กระดาษทิชชู่ PASEO เบบี้เพียว หนา 3 ชั้น สัมผัสนุ่มละมุน อ่อนโยนต่อผิว ยกลังสุดคุ้ม</t>
         </is>
       </c>
     </row>

</xml_diff>